<commit_message>
chore: actualizar dossier y dashboard 2026-05-16
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T53"/>
+  <dimension ref="A1:T44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -567,32 +567,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Desigualdades urbano-ambientales en el marco de la crisis socioecológica. Debates teóricos, metodológicos y políticos</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -647,50 +647,50 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/36</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista de Estudos Aplicados em Educação</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>São Caetano do Sul</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Chamada Dossiê temático: MESTRADO PROFISSIONAL EM EDUCAÇÃO E PRODUTOS EDUCACIONAIS: CONTRIBUIÇÕES PARA O DESENVOLVIMENTO PROFISSIONAL</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -749,46 +749,46 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://seer.uscs.edu.br/index.php/revista_estudos_aplicados/pt_BR/announcement/view/77</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
@@ -854,14 +854,14 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Campos en Ciencias Sociales</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -881,12 +881,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>abierta (2027-I) | Investigación creación | Campos en Ciencias Sociales</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -941,50 +941,50 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S5" t="n">
         <v>74</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://revistas.usantotomas.edu.co/index.php/campos/announcement/view/152</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1039,25 +1039,25 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>74</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1067,22 +1067,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>TEMÁTICO - Privatización de la educación en América Latina: Temas y contenido de las propuestas</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1132,30 +1132,30 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="S7" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2067</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Revista de Estudos Aplicados em Educação</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1165,22 +1165,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>São Caetano do Sul</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Chamada Dossiê temático: MESTRADO PROFISSIONAL EM EDUCAÇÃO E PRODUTOS EDUCACIONAIS: CONTRIBUIÇÕES PARA O DESENVOLVIMENTO PROFISSIONAL</t>
+          <t>TEMÁTICO - Tiempos y espacios escolares en disputa. Debates contemporáneos en el campo pedagógico</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1230,55 +1230,55 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://seer.uscs.edu.br/index.php/revista_estudos_aplicados/pt_BR/announcement/view/77</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2124</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1328,55 +1328,55 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="S9" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1426,55 +1426,55 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Campos en Ciencias Sociales</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>abierta (2027-I) | Investigación creación | Campos en Ciencias Sociales</t>
+          <t>Oportunidad para participar en Revista Científica de Lectura y Escritura</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1524,23 +1524,23 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="S11" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.usantotomas.edu.co/index.php/campos/announcement/view/152</t>
+          <t>https://educacion.uncuyo.edu.ar/oportunidad-para-participar-en-revista-cientifica-de-lectura-y-escritura</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>TEMÁTICO - Privatización de la educación en América Latina: Temas y contenido de las propuestas</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1622,55 +1622,55 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>71</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2067</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TEMÁTICO - Tiempos y espacios escolares en disputa. Debates contemporáneos en el campo pedagógico</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1725,50 +1725,50 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="S13" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2124</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1778,12 +1778,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1823,40 +1823,40 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>46</v>
+        <v>152</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1921,40 +1921,40 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="S15" t="n">
         <v>68</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Oportunidad para participar en Revista Científica de Lectura y Escritura</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2019,18 +2019,18 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/oportunidad-para-participar-en-revista-cientifica-de-lectura-y-escritura</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
@@ -2057,12 +2057,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2117,25 +2117,25 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="S17" t="n">
         <v>68</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/announcement</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -2155,12 +2155,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2215,25 +2215,25 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>97</v>
+        <v>230</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2253,12 +2253,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2313,45 +2313,45 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R19" t="n">
-        <v>153</v>
+        <v>230</v>
       </c>
       <c r="S19" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2415,36 +2415,36 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2513,21 +2513,21 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="S21" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2611,21 +2611,21 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2709,21 +2709,21 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="S23" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2743,12 +2743,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2803,40 +2803,40 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>231</v>
+        <v>325</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>63</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2901,50 +2901,50 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>231</v>
+        <v>345</v>
       </c>
       <c r="S25" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/en_US?source=%2Findex.php%2FRCHP%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2999,50 +2999,50 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>231</v>
+        <v>345</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/pt_BR?source=%2Findex.php%2FRCHP%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3052,12 +3052,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3097,25 +3097,25 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R27" t="n">
-        <v>231</v>
+        <v>345</v>
       </c>
       <c r="S27" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/294</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3135,12 +3135,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3195,50 +3195,50 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>326</v>
+        <v>355</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3248,12 +3248,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3293,50 +3293,50 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="S29" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/en_US?source=%2Findex.php%2FRCHP%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3346,12 +3346,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3391,50 +3391,50 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/pt_BR?source=%2Findex.php%2FRCHP%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3444,12 +3444,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3489,50 +3489,50 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="S31" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/294</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3542,12 +3542,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -3572,40 +3572,42 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
-        </is>
-      </c>
-      <c r="R32" s="2" t="n">
-        <v>351</v>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S32" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/forum/about/submissions</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3617,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3627,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3640,12 +3642,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3670,40 +3672,42 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
-        </is>
-      </c>
-      <c r="R33" t="n">
-        <v>356</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S33" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3717,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3727,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3742,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3768,40 +3772,42 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
-        </is>
-      </c>
-      <c r="R34" s="2" t="n">
-        <v>356</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S34" s="2" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3811,7 +3817,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3821,12 +3827,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3836,12 +3842,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3866,65 +3872,67 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
-        </is>
-      </c>
-      <c r="R35" t="n">
-        <v>356</v>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S35" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3934,12 +3942,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3964,65 +3972,67 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
-        </is>
-      </c>
-      <c r="R36" s="2" t="n">
-        <v>365</v>
+          <t>2027-02-15</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S36" s="2" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Cierre de la  2026</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4032,12 +4042,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -4062,65 +4072,67 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2076-05-15</t>
-        </is>
-      </c>
-      <c r="R37" t="n">
-        <v>18263</v>
+          <t>2027-04-26</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S37" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/432</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4175,7 +4187,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>5000-05-01</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4184,18 +4196,18 @@
         </is>
       </c>
       <c r="S38" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4205,7 +4217,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4215,12 +4227,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4275,7 +4287,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4288,14 +4300,14 @@
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4305,7 +4317,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -4315,12 +4327,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4375,7 +4387,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4388,14 +4400,14 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4405,7 +4417,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4415,7 +4427,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4430,12 +4442,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4475,7 +4487,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4484,43 +4496,43 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4575,7 +4587,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4584,18 +4596,18 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/forum/announcement</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Quid 16</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4615,12 +4627,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16//view/78</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4655,7 +4667,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -4675,7 +4687,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4688,14 +4700,14 @@
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/about/submissions</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/announcement/view/78</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4705,7 +4717,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4715,12 +4727,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4730,12 +4742,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4775,7 +4787,7 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
@@ -4784,909 +4796,9 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
-        <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/about/submissions</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Revista Exitus</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Santarém</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>educación, política</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Anúncios</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>2027-02-15</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S45" t="n">
-        <v>55</v>
-      </c>
-      <c r="T45" s="4" t="inlineStr">
-        <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Revista Chilena de Pedagogía</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Santiago</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Cierre de la  2026</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>2027-04-26</t>
-        </is>
-      </c>
-      <c r="R46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S46" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="T46" s="3" t="inlineStr">
-        <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/432</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Envíos</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>5000-05-01</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S47" t="n">
-        <v>67</v>
-      </c>
-      <c r="T47" s="4" t="inlineStr">
-        <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Revista de educación (Mar del Plata)</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Mar del Plata</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>educación, sociología, política, humanidades</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="T48" s="3" t="inlineStr">
-        <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Raigal</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Villa María</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>sociología, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S49" t="n">
-        <v>70</v>
-      </c>
-      <c r="T49" s="4" t="inlineStr">
-        <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Delito y Sociedad</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>sociología, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P50" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S50" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="T50" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S51" t="n">
-        <v>64</v>
-      </c>
-      <c r="T51" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Quid 16</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>sociología, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16//view/78</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M52" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N52" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O52" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P52" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S52" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="T52" s="3" t="inlineStr">
-        <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/announcement/view/78</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S53" t="n">
-        <v>57</v>
-      </c>
-      <c r="T53" s="4" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5737,15 +4849,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T53" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-05-20
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T50"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -665,32 +665,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -745,50 +745,50 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista de Estudos Aplicados em Educação</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>São Caetano do Sul</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Chamada Dossiê temático: MESTRADO PROFISSIONAL EM EDUCAÇÃO E PRODUTOS EDUCACIONAIS: CONTRIBUIÇÕES PARA O DESENVOLVIMENTO PROFISSIONAL</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -847,46 +847,46 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://seer.uscs.edu.br/index.php/revista_estudos_aplicados/pt_BR/announcement/view/77</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>TEMÁTICO - Privatización de la educación en América Latina: Temas y contenido de las propuestas</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -936,55 +936,55 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="S5" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2067</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>TEMÁTICO - Tiempos y espacios escolares en disputa. Debates contemporáneos en el campo pedagógico</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1034,55 +1034,55 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2124</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1132,30 +1132,30 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="S7" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://seer.ufrgs.br/poled</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1165,22 +1165,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1230,55 +1230,55 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Revista de Estudos Aplicados em Educação</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>São Caetano do Sul</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Chamada Dossiê temático: MESTRADO PROFISSIONAL EM EDUCAÇÃO E PRODUTOS EDUCACIONAIS: CONTRIBUIÇÕES PARA O DESENVOLVIMENTO PROFISSIONAL</t>
+          <t>Oportunidad para participar en Revista Científica de Lectura y Escritura</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1328,23 +1328,23 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="S9" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://seer.uscs.edu.br/index.php/revista_estudos_aplicados/pt_BR/announcement/view/77</t>
+          <t>https://educacion.uncuyo.edu.ar/oportunidad-para-participar-en-revista-cientifica-de-lectura-y-escritura</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>TEMÁTICO - Privatización de la educación en América Latina: Temas y contenido de las propuestas</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1426,55 +1426,55 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>71</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2067</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/announcement</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TEMÁTICO - Tiempos y espacios escolares en disputa. Debates contemporáneos en el campo pedagógico</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1529,50 +1529,50 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="S11" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/announcement/view/2124</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Quid 16</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1627,50 +1627,50 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>42</v>
+        <v>121</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/announcement</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Quid 16</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1725,25 +1725,25 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>42</v>
+        <v>121</v>
       </c>
       <c r="S13" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/poled#homepageAnnouncements</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Oportunidad para participar en Revista Científica de Lectura y Escritura</t>
+          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1778,12 +1778,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1823,18 +1823,18 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>42</v>
+        <v>148</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/oportunidad-para-participar-en-revista-cientifica-de-lectura-y-escritura</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
         </is>
       </c>
     </row>
@@ -1861,12 +1861,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1921,25 +1921,25 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>42</v>
+        <v>226</v>
       </c>
       <c r="S15" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/announcement</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2019,25 +2019,25 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>93</v>
+        <v>226</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2057,12 +2057,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2117,50 +2117,50 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>149</v>
+        <v>226</v>
       </c>
       <c r="S17" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Revista Latinoamericana de Estudios Educativos</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Manizales</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Envíos | Latinoamericana de Estudios Educativos</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2170,12 +2170,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -2219,36 +2219,36 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2268,12 +2268,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2317,21 +2317,21 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="S19" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2415,21 +2415,21 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2513,21 +2513,21 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="S21" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2547,12 +2547,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2607,40 +2607,40 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>227</v>
+        <v>321</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>63</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2705,50 +2705,50 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R23" t="n">
-        <v>227</v>
+        <v>341</v>
       </c>
       <c r="S23" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/en_US?source=%2Findex.php%2FRCHP%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2758,12 +2758,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2803,50 +2803,50 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>227</v>
+        <v>341</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/pt_BR?source=%2Findex.php%2FRCHP%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2901,40 +2901,40 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>227</v>
+        <v>341</v>
       </c>
       <c r="S25" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/294</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Forum. Revista Departamento de Ciencia Política</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>Forum. Revista Departamento de Ciencia Política</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2999,45 +2999,45 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-05-01</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>322</v>
+        <v>346</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://revistas.unal.edu.co/index.php/forum/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3052,12 +3052,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3097,45 +3097,45 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R27" t="n">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="S27" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/en_US?source=%2Findex.php%2FRCHP%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3150,12 +3150,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3195,50 +3195,50 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/pt_BR?source=%2Findex.php%2FRCHP%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3248,12 +3248,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3293,50 +3293,50 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="S29" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/294</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3346,12 +3346,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3391,25 +3391,25 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/forum/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3444,12 +3444,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3489,25 +3489,25 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-05-20</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="S31" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3587,25 +3587,25 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2076-05-20</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>352</v>
+        <v>18263</v>
       </c>
       <c r="S32" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3625,12 +3625,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3685,25 +3685,25 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2110-05-22</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>352</v>
+        <v>30682</v>
       </c>
       <c r="S33" t="n">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3768,40 +3768,42 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
-        </is>
-      </c>
-      <c r="R34" s="2" t="n">
-        <v>361</v>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S34" s="2" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3811,7 +3813,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3821,12 +3823,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3836,12 +3838,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3866,40 +3868,42 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2076-05-19</t>
-        </is>
-      </c>
-      <c r="R35" t="n">
-        <v>18263</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S35" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3909,7 +3913,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3919,12 +3923,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3964,40 +3968,42 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2110-05-22</t>
-        </is>
-      </c>
-      <c r="R36" s="2" t="n">
-        <v>30683</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S36" s="2" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Forum. Revista Departamento de Ciencia Política</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4007,7 +4013,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Bogotá</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -4022,7 +4028,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Forum. Revista Departamento de Ciencia Política</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4077,7 +4083,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -4090,14 +4096,14 @@
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
+          <t>https://revistas.unal.edu.co/index.php/forum/announcement</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -4117,12 +4123,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4177,7 +4183,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -4190,14 +4196,14 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://www.saiehe.org.ar/anuario/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4207,7 +4213,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4217,12 +4223,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4277,7 +4283,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4286,43 +4292,43 @@
         </is>
       </c>
       <c r="S39" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4377,7 +4383,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
@@ -4386,43 +4392,43 @@
         </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>Cierre de la  2026</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4477,7 +4483,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4490,14 +4496,14 @@
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/forum/announcement</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/432</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4517,7 +4523,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -4532,12 +4538,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4577,7 +4583,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>5000-05-01</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4586,43 +4592,43 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/about/submissions</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4632,12 +4638,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4677,7 +4683,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4686,43 +4692,43 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Cierre de la  2026</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4777,7 +4783,7 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
@@ -4790,14 +4796,14 @@
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/432</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4807,7 +4813,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4817,12 +4823,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4832,12 +4838,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4877,7 +4883,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>5000-05-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4886,18 +4892,18 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4907,7 +4913,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -4917,12 +4923,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4986,18 +4992,18 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5017,7 +5023,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5086,309 +5092,9 @@
         </is>
       </c>
       <c r="S47" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="T47" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="T48" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Quid 16</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>sociología, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16//view/78</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S49" t="n">
-        <v>78</v>
-      </c>
-      <c r="T49" s="4" t="inlineStr">
-        <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/announcement/view/78</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P50" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S50" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="T50" s="3" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5442,9 +5148,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-06-03
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T53"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>74</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
         <v>64</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>59</v>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S5" t="n">
         <v>71</v>
@@ -979,7 +979,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1043,10 +1043,10 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S7" t="n">
         <v>71</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>71</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S9" t="n">
         <v>71</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>71</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S11" t="n">
         <v>71</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>71</v>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="R13" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="S15" t="n">
         <v>71</v>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>71</v>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="S17" t="n">
         <v>71</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>71</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="S19" t="n">
         <v>76</v>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S20" s="2" t="n">
         <v>76</v>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S21" t="n">
         <v>70</v>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="S22" s="2" t="n">
         <v>76</v>
@@ -2625,22 +2625,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Políticas Educativas – PolEd</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mercosur</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2709,41 +2709,41 @@
         </is>
       </c>
       <c r="R23" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="S23" t="n">
         <v>68</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2758,12 +2758,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2807,21 +2807,21 @@
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2905,21 +2905,21 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="S25" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -3003,21 +3003,21 @@
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3101,21 +3101,21 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="S27" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3199,21 +3199,21 @@
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3297,21 +3297,21 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="S29" t="n">
         <v>55</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3391,50 +3391,50 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>308</v>
+        <v>212</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3444,12 +3444,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3489,50 +3489,50 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>328</v>
+        <v>307</v>
       </c>
       <c r="S31" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/en_US?source=%2Findex.php%2FRCHP%2Fannouncement</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3542,12 +3542,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -3587,45 +3587,45 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="S32" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/pt_BR?source=%2Findex.php%2FRCHP%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3685,50 +3685,50 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="S33" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/294</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3783,25 +3783,25 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/forum/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3821,12 +3821,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3881,25 +3881,25 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="S35" t="n">
         <v>76</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3919,12 +3919,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3979,25 +3979,25 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2076-06-03</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
-        <v>338</v>
+        <v>18263</v>
       </c>
       <c r="S36" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -4017,12 +4017,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4032,12 +4032,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -4077,25 +4077,25 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2027-05-06</t>
+          <t>2110-05-22</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>338</v>
+        <v>30668</v>
       </c>
       <c r="S37" t="n">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -4115,12 +4115,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4130,12 +4130,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -4160,40 +4160,42 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
-        </is>
-      </c>
-      <c r="R38" s="2" t="n">
-        <v>347</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S38" s="2" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Historia de la Educación. Anuario</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4203,7 +4205,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4213,12 +4215,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4228,12 +4230,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4258,40 +4260,42 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2076-06-02</t>
-        </is>
-      </c>
-      <c r="R39" t="n">
-        <v>18263</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S39" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://www.saiehe.org.ar/anuario/revista/announcement</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4301,7 +4305,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -4311,12 +4315,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4356,65 +4360,67 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2110-05-22</t>
-        </is>
-      </c>
-      <c r="R40" s="2" t="n">
-        <v>30669</v>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S40" s="2" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/categorias/index/convocatorias</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Del prudente Saber</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4469,7 +4475,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2027-02-15</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4478,18 +4484,18 @@
         </is>
       </c>
       <c r="S41" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4499,7 +4505,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -4514,7 +4520,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4569,7 +4575,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>5000-06-01</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
@@ -4578,43 +4584,43 @@
         </is>
       </c>
       <c r="S42" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4624,12 +4630,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4669,7 +4675,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4678,18 +4684,18 @@
         </is>
       </c>
       <c r="S43" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/forum/announcement</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Contextos de Educación</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4699,7 +4705,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Río Cuarto</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4709,12 +4715,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4769,7 +4775,7 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
@@ -4778,43 +4784,43 @@
         </is>
       </c>
       <c r="S44" s="2" t="n">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/about/submissions</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Revista Exitus</t>
+          <t>Historia de la Educación. Anuario</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Anuario de Historia de la Educación</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4824,12 +4830,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4869,7 +4875,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>2027-02-15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4878,43 +4884,43 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
+          <t>https://www.saiehe.org.ar/anuario/revista</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Cierre de la  2026</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4924,12 +4930,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4969,7 +4975,7 @@
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr">
@@ -4978,18 +4984,18 @@
         </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/432</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4999,7 +5005,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5009,12 +5015,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5069,7 +5075,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>5000-06-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -5078,18 +5084,18 @@
         </is>
       </c>
       <c r="S47" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="T47" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -5099,7 +5105,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -5109,12 +5115,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -5178,509 +5184,9 @@
         </is>
       </c>
       <c r="S48" s="2" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="T48" s="3" t="inlineStr">
-        <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Raigal</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Villa María</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>sociología, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S49" t="n">
-        <v>70</v>
-      </c>
-      <c r="T49" s="4" t="inlineStr">
-        <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Historia de la Educación. Anuario</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>Anuario de Historia de la Educación</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P50" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S50" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="T50" s="3" t="inlineStr">
-        <is>
-          <t>https://www.saiehe.org.ar/anuario/revista</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Delito y Sociedad</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>sociología, política, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S51" t="n">
-        <v>78</v>
-      </c>
-      <c r="T51" s="4" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>El Taco en la Brea</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>Para autores</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M52" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N52" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O52" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P52" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S52" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="T52" s="3" t="inlineStr">
-        <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S53" t="n">
-        <v>57</v>
-      </c>
-      <c r="T53" s="4" t="inlineStr">
         <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
         </is>
@@ -5735,11 +5241,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T53" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualizar dossier y dashboard 2026-09-02
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T63"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -567,32 +567,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Políticas Educativas – PolEd</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Mercosur</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -647,50 +647,50 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
+          <t>https://seer.ufrgs.br/index.php/Poled/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Educação em Revista</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Submissão</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -745,50 +745,50 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
+          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -798,12 +798,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -843,50 +843,50 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -896,12 +896,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -941,50 +941,50 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S5" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1039,50 +1039,50 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1092,12 +1092,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1137,50 +1137,50 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S7" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista de Estudos Aplicados em Educação</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>São Caetano do Sul</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Desigualdades urbano-ambientales en el marco de la crisis socioecológica. Debates teóricos, metodológicos y políticos</t>
+          <t>Chamada Dossiê temático: MESTRADO PROFISSIONAL EM EDUCAÇÃO E PRODUTOS EDUCACIONAIS: CONTRIBUIÇÕES PARA O DESENVOLVIMENTO PROFISSIONAL</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1235,25 +1235,25 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/36</t>
+          <t>https://seer.uscs.edu.br/index.php/revista_estudos_aplicados/pt_BR/announcement/view/77</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Quid 16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1328,30 +1328,30 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="S9" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/announcement</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Quid 16</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1371,12 +1371,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>"Educación y arraigo en los territorios rurales de América Latina. Pedagogías colaborativas, re existencias y acciones colectivas para la construcción de futuros viables"</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1426,30 +1426,30 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>próxima</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/30</t>
+          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Revista de educación (Mar del Plata)</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>educación</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/about/submissions#authorGuidelines</t>
+          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1524,55 +1524,55 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="S11" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/about/submissions#authorGuidelines</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía: s</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1622,55 +1622,55 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/gateway/plugin/AnnouncementFeedGatewayPlugin/atom</t>
+          <t>https://revista.saap.org.ar/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Forum. Revista Departamento de Ciencia Política</t>
+          <t>REVISTA SAAP</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1720,30 +1720,30 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="S13" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/forum/about/submissions</t>
+          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1763,12 +1763,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1818,55 +1818,55 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>CLACSO Convocatorias</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Ciudad de México</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Latinoamérica</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>REVISTA SAAP</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1876,12 +1876,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1916,55 +1916,55 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="S15" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/#homepageAnnouncements</t>
+          <t>https://www.clacso.org/publicaciones-convocatorias/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>CLACSO Convocatorias</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Ciudad de México</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latinoamérica</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2014,55 +2014,55 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/about/submissions</t>
+          <t>https://www.clacso.org/publicaciones-convocatorias/#content</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>CLACSO Convocatorias</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Ciudad de México</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Latinoamérica</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>educación, sociología, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>“Estudios críticos de la Gestión. Perspectivas y dimensiones”</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2072,12 +2072,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2112,45 +2112,45 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="S17" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/18</t>
+          <t>https://www.clacso.org/publicaciones-convocatorias/#ekit_modal-popup-27f205e</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Sociohistórica</t>
+          <t>CLACSO Convocatorias</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Ciudad de México</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Latinoamérica</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2170,12 +2170,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -2210,30 +2210,30 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://www.clacso.org/publicaciones-convocatorias/#ekit_modal-popup-bd356d0</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2253,12 +2253,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Prórroga Dossier "El desafío actual de los riesgos psicosociales en el trabajo"</t>
+          <t>a Dossier temático “Políticas públicas y discursos sobre la escuela interpretados desde las prácticas educativas”</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2308,30 +2308,30 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S19" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/24</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2351,12 +2351,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Resultados para ""</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2406,30 +2406,30 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Quid 16</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2449,12 +2449,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16//view/168</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2504,55 +2504,55 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R21" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S21" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/announcement/view/168</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_main</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Educação em Revista</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Submissão</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2602,55 +2602,55 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>https://periodicos.ufmg.br/index.php/edrevista/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#siteNav</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2700,55 +2700,55 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S23" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement#pkp_content_footer</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2758,12 +2758,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2798,55 +2798,55 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#authorGuidelines</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/es_ES?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2896,55 +2896,55 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S25" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#privacyStatement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Historia y Sociedad</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Medellín</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Historia y sociedad</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2994,50 +2994,50 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/about/submissions#onlineSubmissions</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3052,12 +3052,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3092,55 +3092,55 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R27" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="S27" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista Iberoamericana de Educación</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Iberoamérica</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Avisos</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3150,12 +3150,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3190,55 +3190,55 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
+          <t>https://rieoei.org/RIE/announcement</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Manizales</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>educación, sociología, política, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Envíos | Latinoamericana de Estudios Educativos</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3248,12 +3248,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3288,30 +3288,30 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="S29" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
+          <t>https://revistasojs.ucaldas.edu.co/index.php/latinoamericana/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Traslaciones / convocatoria UNCuyo</t>
+          <t>Sociohistórica</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3331,12 +3331,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3346,12 +3346,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3386,30 +3386,30 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>https://educacion.uncuyo.edu.ar/convocatorias-a-becas-y-proyectos-de-investigacion-y-posgrado</t>
+          <t>https://www.sociohistorica.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3484,30 +3484,30 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="S31" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
+          <t>https://revista.saap.org.ar/index.php/revista/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Clío y Asociados</t>
+          <t>Archivos de Ciencias de la Educación</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>La Plata</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3582,55 +3582,55 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="S32" s="2" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
+          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revista de Estudos Aplicados em Educação</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>São Caetano do Sul</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>educación, política</t>
+          <t>educación, sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Chamada Dossiê temático: MESTRADO PROFISSIONAL EM EDUCAÇÃO E PRODUTOS EDUCACIONAIS: CONTRIBUIÇÕES PARA O DESENVOLVIMENTO PROFISSIONAL</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3680,30 +3680,30 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>5</v>
+        <v>121</v>
       </c>
       <c r="S33" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>https://seer.uscs.edu.br/index.php/revista_estudos_aplicados/pt_BR/announcement/view/77</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Quid 16</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -3778,30 +3778,30 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>17</v>
+        <v>121</v>
       </c>
       <c r="S34" s="2" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16/announcement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Quid 16</t>
+          <t>Clío y Asociados</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3821,12 +3821,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3876,30 +3876,30 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>próxima</t>
+          <t>abierta</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="R35" t="n">
-        <v>17</v>
+        <v>121</v>
       </c>
       <c r="S35" t="n">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
-          <t>https://publicaciones.sociales.uba.ar/index.php/quid16</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ClioyAsociados/es/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Archivos de Ciencias de la Educación</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>La Plata</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3919,12 +3919,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>sociología, política</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Agendas emergentes y enfoques situados en los estudios sobre la evaluación académica y de la investigación: introducción al dosier</t>
+          <t>Propuestas de Dossier Temático</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3979,50 +3979,50 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2027-04-06</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
-        <v>28</v>
+        <v>216</v>
       </c>
       <c r="S36" s="2" t="n">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>https://www.archivosdeciencias.fahce.unlp.edu.ar/article/view/Archivose181</t>
+          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>educación, sociología, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>"Experiencias formativas en la pospandemia: avances y desafíos para las carreras universitarias en salud"</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4032,12 +4032,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -4077,45 +4077,45 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R37" t="n">
-        <v>44</v>
+        <v>236</v>
       </c>
       <c r="S37" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="T37" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/34</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/en_US?source=%2Findex.php%2FRCHP%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>CLACSO Convocatorias</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Ciudad de México</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Latinoamérica</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -4175,50 +4175,50 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R38" s="2" t="n">
-        <v>59</v>
+        <v>236</v>
       </c>
       <c r="S38" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>https://www.clacso.org/publicaciones-convocatorias/</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/294</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CLACSO Convocatorias</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Ciudad de México</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Latinoamérica</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4273,50 +4273,50 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2027-04-26</t>
         </is>
       </c>
       <c r="R39" t="n">
-        <v>59</v>
+        <v>236</v>
       </c>
       <c r="S39" t="n">
         <v>68</v>
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>https://www.clacso.org/publicaciones-convocatorias/#content</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/pt_BR?source=%2Findex.php%2FRCHP%2Fannouncement</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>CLACSO Convocatorias</t>
+          <t>Revista Análisis de las Prácticas</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Ciudad de México</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Latinoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, política</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>a Dossier temático “La dimensión colectiva del trabajo docente”</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4326,12 +4326,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -4371,40 +4371,40 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2027-05-06</t>
         </is>
       </c>
       <c r="R40" s="2" t="n">
-        <v>59</v>
+        <v>246</v>
       </c>
       <c r="S40" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>https://www.clacso.org/publicaciones-convocatorias/#ekit_modal-popup-27f205e</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/13</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CLACSO Convocatorias</t>
+          <t>De Prácticas y Discursos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ciudad de México</t>
+          <t>Corrientes</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Latinoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4424,12 +4424,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4469,25 +4469,25 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="R41" t="n">
-        <v>59</v>
+        <v>255</v>
       </c>
       <c r="S41" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>https://www.clacso.org/publicaciones-convocatorias/#ekit_modal-popup-bd356d0</t>
+          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista SAAP</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4507,12 +4507,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4567,18 +4567,18 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-08-15</t>
         </is>
       </c>
       <c r="R42" s="2" t="n">
-        <v>101</v>
+        <v>347</v>
       </c>
       <c r="S42" s="2" t="n">
         <v>76</v>
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/en_US?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
         </is>
       </c>
     </row>
@@ -4605,12 +4605,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>educación, sociología, política</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4665,50 +4665,50 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2027-08-20</t>
         </is>
       </c>
       <c r="R43" t="n">
-        <v>101</v>
+        <v>352</v>
       </c>
       <c r="S43" t="n">
         <v>76</v>
       </c>
       <c r="T43" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/user/setLocale/pt_BR?source=%2Findex.php%2Fanalisispracticas%2Fannouncement</t>
+          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Revista Iberoamericana de Educación</t>
+          <t>Traslaciones / convocatoria UNCuyo</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Iberoamérica</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>educación, política, ciencias sociales</t>
+          <t>educación, sociología, política, humanidades</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Avisos</t>
+          <t>Resultados para ""</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4763,25 +4763,25 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2027-08-24</t>
         </is>
       </c>
       <c r="R44" s="2" t="n">
-        <v>122</v>
+        <v>356</v>
       </c>
       <c r="S44" s="2" t="n">
         <v>68</v>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>https://rieoei.org/RIE/announcement</t>
+          <t>https://educacion.uncuyo.edu.ar/buscar_tag/index/?tag=convocatoria</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Raigal</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4791,7 +4791,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Villa María</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4801,12 +4801,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>sociología, política</t>
+          <t>educación, sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Propuestas de Dossier Temático</t>
+          <t>s</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4816,12 +4816,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4846,65 +4846,67 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>2027-04-06</t>
-        </is>
-      </c>
-      <c r="R45" t="n">
-        <v>217</v>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S45" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/propuestas-dossier</t>
+          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Historia y Sociedad</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Medellín</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>sociología, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Historia y sociedad</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4944,65 +4946,67 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
-        </is>
-      </c>
-      <c r="R46" s="2" t="n">
-        <v>237</v>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S46" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/en_US?source=%2Findex.php%2FRCHP%2Fannouncement</t>
+          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Del prudente Saber</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5042,65 +5046,67 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
-        </is>
-      </c>
-      <c r="R47" t="n">
-        <v>237</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S47" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T47" s="4" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/294</t>
+          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Cuadernos del CIESAL</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Rosario</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Anúncios</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -5140,40 +5146,42 @@
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>2027-04-26</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="n">
-        <v>237</v>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S48" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="T48" s="3" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/user/setLocale/pt_BR?source=%2Findex.php%2FRCHP%2Fannouncement</t>
+          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>De Prácticas y Discursos</t>
+          <t>Contextos de Educación</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5183,7 +5191,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Corrientes</t>
+          <t>Río Cuarto</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5193,12 +5201,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>educación, política, humanidades</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>al Dossier Perspectivas y Desafíos en la Investigación Cualitativa: Método y Experiencias</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -5208,12 +5216,12 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5238,65 +5246,67 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
-        </is>
-      </c>
-      <c r="R49" t="n">
-        <v>256</v>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S49" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="T49" s="4" t="inlineStr">
         <is>
-          <t>https://revistas.unne.edu.ar/index.php/dpd/announcement/view/37</t>
+          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Revista SAAP</t>
+          <t>Revista Exitus</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>educación, política</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>PARA PROPUESTAS DE DOSSIER - REVISTA SAAP</t>
+          <t>Anúncios</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -5306,12 +5316,12 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -5336,65 +5346,67 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="n">
-        <v>348</v>
+          <t>2027-02-15</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S50" s="2" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="T50" s="3" t="inlineStr">
         <is>
-          <t>https://revista.saap.org.ar/index.php/revista/announcement/view/9</t>
+          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Revista Análisis de las Prácticas</t>
+          <t>Revista Chilena de Pedagogía</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Buenos Aires</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades</t>
+          <t>educación, política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>temático. La escuela secundaria: problemas, experiencias y perspectivas</t>
+          <t>Cierre de la  2026</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5404,12 +5416,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -5434,40 +5446,42 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>permanente</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>permanent</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>abierta</t>
+          <t>continua</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>2027-08-20</t>
-        </is>
-      </c>
-      <c r="R51" t="n">
-        <v>353</v>
+          <t>2027-04-26</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="S51" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="T51" s="4" t="inlineStr">
         <is>
-          <t>https://portalrevistas.unipe.edu.ar/index.php/analisispracticas/announcement/view/11</t>
+          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/432</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Raigal</t>
+          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -5477,7 +5491,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Villa María</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -5487,12 +5501,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>educación, sociología, política, humanidades, ciencias sociales</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Envíos</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -5547,7 +5561,7 @@
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>5000-09-01</t>
         </is>
       </c>
       <c r="R52" s="2" t="inlineStr">
@@ -5556,43 +5570,43 @@
         </is>
       </c>
       <c r="S52" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="T52" s="3" t="inlineStr">
         <is>
-          <t>https://raigal.unvm.edu.ar/ojs/index.php/raigal/convocatorias</t>
+          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Revista Chilena de Pedagogía</t>
+          <t>Revista de educación (Mar del Plata)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Mar del Plata</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>educación, política, humanidades, ciencias sociales</t>
+          <t>educación, sociología, humanidades</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Cierre de la  2026</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -5602,12 +5616,12 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5647,7 +5661,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -5656,18 +5670,18 @@
         </is>
       </c>
       <c r="S53" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T53" s="4" t="inlineStr">
         <is>
-          <t>https://revistadepedagogia.uchile.cl/index.php/RCHP/announcement/view/432</t>
+          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Cuadernos del CIESAL</t>
+          <t>Delito y Sociedad</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -5677,7 +5691,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Rosario</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -5687,7 +5701,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades, ciencias sociales</t>
+          <t>sociología, política, ciencias sociales</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -5702,12 +5716,12 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -5747,7 +5761,7 @@
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr">
@@ -5756,18 +5770,18 @@
         </is>
       </c>
       <c r="S54" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="T54" s="3" t="inlineStr">
         <is>
-          <t>https://cuadernosdelciesal.unr.edu.ar/index.php/inicio/about</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Delito y Sociedad</t>
+          <t>El Taco en la Brea</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5787,12 +5801,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>sociología, política, ciencias sociales</t>
+          <t>política, humanidades</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Sobre la revista</t>
+          <t>Para autores</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5802,12 +5816,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>NBRA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>CAICYT-CONICET</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -5847,7 +5861,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5856,18 +5870,18 @@
         </is>
       </c>
       <c r="S55" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="T55" s="4" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DelitoySociedad/about/index</t>
+          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>El Taco en la Brea</t>
+          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -5887,12 +5901,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>política, humanidades</t>
+          <t>política, humanidades, ciencias sociales</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Para autores</t>
+          <t>Sobre la revista</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -5902,12 +5916,12 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NBRA</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CAICYT-CONICET</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -5947,7 +5961,7 @@
       </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R56" s="2" t="inlineStr">
@@ -5956,711 +5970,11 @@
         </is>
       </c>
       <c r="S56" s="2" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="T56" s="3" t="inlineStr">
         <is>
-          <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/ElTacoenlaBrea/autores/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Contextos de Educación</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Río Cuarto</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>educación, política, humanidades</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Envíos</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S57" t="n">
-        <v>59</v>
-      </c>
-      <c r="T57" s="4" t="inlineStr">
-        <is>
-          <t>https://www2.hum.unrc.edu.ar/ojs/index.php/contextos/about/submissions</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Revista Exitus</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Santarém</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>educación, política</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>Anúncios</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M58" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N58" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O58" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P58" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q58" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="R58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S58" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="T58" s="3" t="inlineStr">
-        <is>
-          <t>https://portaldeperiodicos.ufopa.edu.br/index.php/revistaexitus/announcement</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Documentos y Aportes en Administración Pública y Gestión Estatal</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Sobre la revista</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P59" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q59" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S59" t="n">
-        <v>57</v>
-      </c>
-      <c r="T59" s="4" t="inlineStr">
-        <is>
           <t>https://bibliotecavirtual.unl.edu.ar/publicaciones/index.php/DocumentosyAportes/about/index</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Historia y Sociedad</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Medellín</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>sociología, política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>Historia y sociedad</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M60" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N60" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O60" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P60" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q60" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="R60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S60" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="T60" s="3" t="inlineStr">
-        <is>
-          <t>https://revistas.unal.edu.co/index.php/hisysoc/announcement</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Del prudente Saber</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Paraná</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>dirección escolar, educación, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>para la edición N° 18 de la revista “del Prudente saber…”</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O61" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q61" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S61" t="n">
-        <v>70</v>
-      </c>
-      <c r="T61" s="4" t="inlineStr">
-        <is>
-          <t>https://www.fcedu.uner.edu.ar/recepcion-continua-para-la-edicion-n-18-de-la-revista-del-prudente-saber/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Chuy. Revista de Estudios Literarios Latinoamericanos</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>política, humanidades, ciencias sociales</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>Envíos</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M62" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N62" s="2" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O62" s="2" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P62" s="2" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q62" s="2" t="inlineStr">
-        <is>
-          <t>5000-09-01</t>
-        </is>
-      </c>
-      <c r="R62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S62" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="T62" s="3" t="inlineStr">
-        <is>
-          <t>https://revistas.untref.edu.ar/index.php/chuy/about/submissions</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Revista de educación (Mar del Plata)</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Mar del Plata</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>educación, sociología, humanidades</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>NBRA</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>CAICYT-CONICET</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>permanente</t>
-        </is>
-      </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t>permanent</t>
-        </is>
-      </c>
-      <c r="P63" t="inlineStr">
-        <is>
-          <t>continua</t>
-        </is>
-      </c>
-      <c r="Q63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S63" t="n">
-        <v>78</v>
-      </c>
-      <c r="T63" s="4" t="inlineStr">
-        <is>
-          <t>https://fh.mdp.edu.ar/revistas/index.php/r_educ/index</t>
         </is>
       </c>
     </row>
@@ -6721,13 +6035,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>